<commit_message>
운동프로그램 갱신 2026-09-07  0:47:06.66
</commit_message>
<xml_diff>
--- a/운동프로그램_10일주기_v19.xlsx
+++ b/운동프로그램_10일주기_v19.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b2bc197408547891/Desktop/운동/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="569" documentId="11_56CBE09B577CB57806506320C7833877887CCA2D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6628712A-9782-40EA-8F3D-F8BBE07F82EC}"/>
+  <xr:revisionPtr revIDLastSave="573" documentId="11_56CBE09B577CB57806506320C7833877887CCA2D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F78A285-37AE-49D5-82CA-3AF2FCC32E0D}"/>
   <bookViews>
-    <workbookView xWindow="6360" yWindow="2400" windowWidth="29040" windowHeight="18480" tabRatio="883" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6360" yWindow="2400" windowWidth="29040" windowHeight="18480" tabRatio="883" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="시작중량_설정" sheetId="1" r:id="rId1"/>
@@ -17476,7 +17476,7 @@
         <v>246</v>
       </c>
       <c r="D6" s="26">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="E6" s="20">
         <v>5</v>
@@ -17516,7 +17516,7 @@
         <v>238</v>
       </c>
       <c r="D7" s="26">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="E7" s="20">
         <v>3</v>
@@ -17722,7 +17722,7 @@
         <v>348</v>
       </c>
       <c r="D12" s="20">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E12" s="20">
         <v>4</v>
@@ -17800,7 +17800,7 @@
         <v>60</v>
       </c>
       <c r="D14" s="26">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E14" s="20">
         <v>3</v>

</xml_diff>

<commit_message>
운동프로그램 갱신 2026-09-14 19:22:58.53
</commit_message>
<xml_diff>
--- a/운동프로그램_10일주기_v19.xlsx
+++ b/운동프로그램_10일주기_v19.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b2bc197408547891/Desktop/운동/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1785" documentId="11_56CBE09B577CB57806506320C7833877887CCA2D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40995B9D-56C0-4BDF-9311-63320D14914C}"/>
+  <xr:revisionPtr revIDLastSave="1796" documentId="11_56CBE09B577CB57806506320C7833877887CCA2D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{177FC5C0-44DB-4791-AFB9-60D7074769CD}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="976" activeTab="17" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="976" activeTab="21" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="시작중량_설정" sheetId="1" r:id="rId1"/>
@@ -11448,7 +11448,7 @@
       </c>
       <c r="E6" s="71">
         <f>복귀_평일A_가슴!$E$28</f>
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F6" s="73" t="s">
         <v>1253</v>
@@ -11472,7 +11472,7 @@
       </c>
       <c r="E7" s="7">
         <f>복귀_평일B_어깨!$E$21</f>
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F7" s="69" t="s">
         <v>1253</v>
@@ -11561,7 +11561,7 @@
       <c r="D11" s="67"/>
       <c r="E11" s="7">
         <f>SUM(E6:E10)</f>
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="F11" s="53" t="s">
         <v>1304</v>
@@ -13639,7 +13639,7 @@
         <v>8</v>
       </c>
       <c r="E12" s="7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F12" s="8" t="s">
         <v>19</v>
@@ -13652,7 +13652,7 @@
       </c>
       <c r="I12">
         <f t="shared" si="0"/>
-        <v>7.7</v>
+        <v>6</v>
       </c>
       <c r="J12" t="s">
         <v>1054</v>
@@ -13678,7 +13678,7 @@
         <v>763</v>
       </c>
       <c r="E13" s="7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F13" s="8" t="s">
         <v>19</v>
@@ -13691,7 +13691,7 @@
       </c>
       <c r="I13">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J13" t="s">
         <v>764</v>
@@ -13962,11 +13962,11 @@
       </c>
       <c r="E21">
         <f>SUM(E11:E20)</f>
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="I21">
         <f>ROUND(SUM(I11:I20),0)</f>
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="22" spans="1:14" ht="237.75" customHeight="1">
@@ -14343,7 +14343,7 @@
         <v>1325</v>
       </c>
       <c r="E22" s="7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F22" s="8" t="s">
         <v>279</v>
@@ -14356,7 +14356,7 @@
       </c>
       <c r="I22">
         <f t="shared" si="0"/>
-        <v>9.6999999999999993</v>
+        <v>7.3</v>
       </c>
       <c r="J22" t="s">
         <v>795</v>
@@ -14415,7 +14415,7 @@
         <v>125</v>
       </c>
       <c r="E24" s="7">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F24" s="8" t="s">
         <v>40</v>
@@ -14428,7 +14428,7 @@
       </c>
       <c r="I24">
         <f>IF(E24=0,0,ROUND((E24*(G24+H24)+N24)/60,1))</f>
-        <v>13.3</v>
+        <v>8</v>
       </c>
       <c r="J24" t="s">
         <v>1308</v>
@@ -14451,7 +14451,7 @@
         <v>125</v>
       </c>
       <c r="E25" s="7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F25" s="8" t="s">
         <v>40</v>
@@ -14464,7 +14464,7 @@
       </c>
       <c r="I25">
         <f t="shared" si="0"/>
-        <v>11.7</v>
+        <v>9</v>
       </c>
       <c r="J25" t="s">
         <v>1310</v>
@@ -14557,11 +14557,11 @@
       </c>
       <c r="E28">
         <f>SUM(E20:E27)</f>
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="I28">
         <f>ROUND(SUM(I20:I27),0)</f>
-        <v>76</v>
+        <v>65</v>
       </c>
     </row>
     <row r="29" spans="1:14" ht="32.25" customHeight="1">
@@ -15887,11 +15887,11 @@
       </c>
       <c r="E8">
         <f t="shared" ca="1" si="0"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F8">
         <f t="shared" ca="1" si="1"/>
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="G8" t="s">
         <v>457</v>
@@ -16559,11 +16559,11 @@
       </c>
       <c r="E32">
         <f t="shared" ca="1" si="2"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F32">
         <f t="shared" ca="1" si="3"/>
-        <v>0.8</v>
+        <v>0.60000000000000009</v>
       </c>
       <c r="G32" t="s">
         <v>457</v>
@@ -17063,11 +17063,11 @@
       </c>
       <c r="E50">
         <f ca="1">IFERROR(INDEX(INDIRECT("'"&amp;$A50&amp;"'!$E$1:$E$45"),MATCH($B50,INDIRECT("'"&amp;$A50&amp;"'!$B$1:$B$45"),0)),"?")</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F50">
         <f ca="1">IF(ISNUMBER(E50),$D50*E50,0)</f>
-        <v>1</v>
+        <v>0.60000000000000009</v>
       </c>
       <c r="G50" t="s">
         <v>457</v>
@@ -17091,11 +17091,11 @@
       </c>
       <c r="E51">
         <f ca="1">IFERROR(INDEX(INDIRECT("'"&amp;$A51&amp;"'!$E$1:$E$45"),MATCH($B51,INDIRECT("'"&amp;$A51&amp;"'!$B$1:$B$45"),0)),"?")</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F51">
         <f ca="1">IF(ISNUMBER(E51),$D51*E51,0)</f>
-        <v>1</v>
+        <v>0.60000000000000009</v>
       </c>
       <c r="G51" t="s">
         <v>457</v>
@@ -17119,11 +17119,11 @@
       </c>
       <c r="E52">
         <f t="shared" ca="1" si="2"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F52">
         <f t="shared" ca="1" si="3"/>
-        <v>0.8</v>
+        <v>0.60000000000000009</v>
       </c>
       <c r="G52" t="s">
         <v>457</v>
@@ -17287,11 +17287,11 @@
       </c>
       <c r="E58">
         <f t="shared" ca="1" si="2"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F58">
         <f t="shared" ca="1" si="3"/>
-        <v>0.8</v>
+        <v>0.60000000000000009</v>
       </c>
       <c r="G58" t="s">
         <v>457</v>
@@ -17375,7 +17375,7 @@
       </c>
       <c r="B5">
         <f>SUMIFS(복귀_평일A_가슴!$E:$E,복귀_평일A_가슴!$C:$C,$A5)+SUMIFS(복귀_평일B_어깨!$E:$E,복귀_평일B_어깨!$C:$C,$A5)+SUMIFS(복귀_토_하체!$E:$E,복귀_토_하체!$C:$C,$A5)+SUMIFS(복귀_일_등!$E:$E,복귀_일_등!$C:$C,$A5)</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C5">
         <f ca="1">MROUND(SUMIFS(복귀_간접계수맵!$F$7:$F$58,복귀_간접계수맵!$C$7:$C$58,$A5),0.5)</f>
@@ -17383,11 +17383,11 @@
       </c>
       <c r="D5">
         <f t="shared" ref="D5:D24" ca="1" si="0">B5+C5</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E5" t="str">
         <f t="shared" ref="E5:E24" ca="1" si="1">IF(D5&gt;20,"과다 점검",IF(D5&gt;=10,"충분",IF(D5&gt;=8,"하한",IF(D5&gt;=1,"보완 필요","미배치"))))</f>
-        <v>충분</v>
+        <v>하한</v>
       </c>
       <c r="F5" t="s">
         <v>1240</v>
@@ -17400,7 +17400,7 @@
       </c>
       <c r="I5">
         <f ca="1">SUM(D5:D6)</f>
-        <v>27.5</v>
+        <v>26.5</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -17436,7 +17436,7 @@
       </c>
       <c r="B7">
         <f>SUMIFS(복귀_평일A_가슴!$E:$E,복귀_평일A_가슴!$C:$C,$A7)+SUMIFS(복귀_평일B_어깨!$E:$E,복귀_평일B_어깨!$C:$C,$A7)+SUMIFS(복귀_토_하체!$E:$E,복귀_토_하체!$C:$C,$A7)+SUMIFS(복귀_일_등!$E:$E,복귀_일_등!$C:$C,$A7)</f>
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C7">
         <f ca="1">MROUND(SUMIFS(복귀_간접계수맵!$F$7:$F$58,복귀_간접계수맵!$C$7:$C$58,$A7),0.5)</f>
@@ -17444,11 +17444,11 @@
       </c>
       <c r="D7">
         <f t="shared" ca="1" si="0"/>
-        <v>21.5</v>
+        <v>18.5</v>
       </c>
       <c r="E7" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>과다 점검</v>
+        <v>충분</v>
       </c>
       <c r="F7" t="s">
         <v>1321</v>
@@ -17461,7 +17461,7 @@
       </c>
       <c r="I7">
         <f ca="1">SUM(D7:D10)</f>
-        <v>45.5</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -17501,11 +17501,11 @@
       </c>
       <c r="C9">
         <f ca="1">MROUND(SUMIFS(복귀_간접계수맵!$F$7:$F$58,복귀_간접계수맵!$C$7:$C$58,$A9),0.5)</f>
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="D9">
         <f t="shared" ca="1" si="0"/>
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="E9" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -17605,7 +17605,7 @@
       </c>
       <c r="B13">
         <f>SUMIFS(복귀_평일A_가슴!$E:$E,복귀_평일A_가슴!$C:$C,$A13)+SUMIFS(복귀_평일B_어깨!$E:$E,복귀_평일B_어깨!$C:$C,$A13)+SUMIFS(복귀_토_하체!$E:$E,복귀_토_하체!$C:$C,$A13)+SUMIFS(복귀_일_등!$E:$E,복귀_일_등!$C:$C,$A13)</f>
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C13">
         <f ca="1">MROUND(SUMIFS(복귀_간접계수맵!$F$7:$F$58,복귀_간접계수맵!$C$7:$C$58,$A13),0.5)</f>
@@ -17613,7 +17613,7 @@
       </c>
       <c r="D13">
         <f t="shared" ca="1" si="0"/>
-        <v>13.5</v>
+        <v>11.5</v>
       </c>
       <c r="E13" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -17805,11 +17805,11 @@
       </c>
       <c r="C20">
         <f ca="1">MROUND(SUMIFS(복귀_간접계수맵!$F$7:$F$58,복귀_간접계수맵!$C$7:$C$58,$A20),0.5)</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D20">
         <f t="shared" ca="1" si="0"/>
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E20" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -17936,11 +17936,11 @@
       </c>
       <c r="B25">
         <f>SUM(B5:B24)</f>
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="D25">
         <f ca="1">SUM(D5:D24)</f>
-        <v>204.5</v>
+        <v>197</v>
       </c>
     </row>
     <row r="27" spans="1:7">

</xml_diff>